<commit_message>
feat(rag-stream): streamline general and ragflow logging
</commit_message>
<xml_diff>
--- a/scripts/岱山-指令集-固定问题 -测试问题0311.xlsx
+++ b/scripts/岱山-指令集-固定问题 -测试问题0311.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
   <si>
     <t>问题</t>
   </si>
@@ -95,6 +95,15 @@
     <t>园区2025年工业总产值</t>
   </si>
   <si>
+    <t>园区2025年规上工业总产值</t>
+  </si>
+  <si>
+    <t>园区2025年亩均产值</t>
+  </si>
+  <si>
+    <t>园区2025年亩均税收</t>
+  </si>
+  <si>
     <t>园区规划面积</t>
   </si>
   <si>
@@ -107,7 +116,7 @@
     <t>园区2025年9月风险走势情况</t>
   </si>
   <si>
-    <t>某企业2025年9月风险走势情况</t>
+    <t>润和催化材料(浙江)有限公司2025年9月风险走势情况</t>
   </si>
   <si>
     <t>园区当前的风险分级管控情况</t>
@@ -414,12 +423,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -738,7 +753,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -762,16 +777,16 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -780,90 +795,91 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1320,283 +1336,283 @@
       </c>
     </row>
     <row r="21" spans="1:1">
-      <c r="A21" t="s">
+      <c r="A21" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="22" spans="1:1">
-      <c r="A22" t="s">
-        <v>21</v>
+      <c r="A22" s="1" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="23" spans="1:1">
-      <c r="A23" t="s">
-        <v>21</v>
+      <c r="A23" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="24" spans="1:1">
-      <c r="A24" t="s">
-        <v>21</v>
+      <c r="A24" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="26" spans="1:1">
       <c r="A26" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="27" spans="1:1">
       <c r="A27" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="28" spans="1:1">
       <c r="A28" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="29" spans="1:1">
       <c r="A29" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="30" spans="1:1">
       <c r="A30" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="31" spans="1:1">
       <c r="A31" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="32" spans="1:1">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="34" spans="1:1">
       <c r="A34" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="35" spans="1:1">
       <c r="A35" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="36" spans="1:1">
       <c r="A36" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="37" spans="1:1">
       <c r="A37" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="38" spans="1:1">
       <c r="A38" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="39" spans="1:1">
       <c r="A39" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="40" spans="1:1">
       <c r="A40" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="41" spans="1:1">
       <c r="A41" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="42" spans="1:1">
       <c r="A42" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="43" spans="1:1">
       <c r="A43" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="44" spans="1:1">
       <c r="A44" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="45" spans="1:1">
       <c r="A45" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="46" spans="1:1">
       <c r="A46" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="47" spans="1:1">
       <c r="A47" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="48" spans="1:1">
       <c r="A48" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="49" spans="1:1">
       <c r="A49" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="50" spans="1:1">
       <c r="A50" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="51" spans="1:1">
       <c r="A51" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="52" spans="1:1">
       <c r="A52" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="53" spans="1:1">
       <c r="A53" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="54" spans="1:1">
       <c r="A54" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="55" spans="1:1">
       <c r="A55" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="56" spans="1:1">
       <c r="A56" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="57" spans="1:1">
       <c r="A57" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="58" spans="1:1">
       <c r="A58" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="59" spans="1:1">
       <c r="A59" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="60" spans="1:1">
       <c r="A60" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="61" spans="1:1">
       <c r="A61" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="62" spans="1:1">
       <c r="A62" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="63" spans="1:1">
       <c r="A63" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="64" spans="1:1">
       <c r="A64" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="65" spans="1:1">
       <c r="A65" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="66" spans="1:1">
       <c r="A66" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="67" spans="1:1">
       <c r="A67" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="68" spans="1:1">
       <c r="A68" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="69" spans="1:1">
       <c r="A69" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="70" spans="1:1">
       <c r="A70" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="71" spans="1:1">
       <c r="A71" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="72" spans="1:1">
       <c r="A72" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="73" spans="1:1">
       <c r="A73" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="74" spans="1:1">
       <c r="A74" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="75" spans="1:1">
       <c r="A75" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="76" spans="1:1">
       <c r="A76" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>